<commit_message>
fix: urutan elemen OOXML (conditionalFormatting sebelum dataValidations) supaya sheet Input Barang tidak di-strip Excel saat open
</commit_message>
<xml_diff>
--- a/Sistem_Keluar_Masuk_Barang.xlsx
+++ b/Sistem_Keluar_Masuk_Barang.xlsx
@@ -9180,16 +9180,16 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B1000">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>COUNTIF($B$2:$B$1000,B2)&gt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="0" showErrorMessage="1" errorStyle="stop" errorTitle="Kode Duplikat" error="Kode barang ini SUDAH ADA di Input. Gunakan kode lain." sqref="B2:B1000">
       <formula1>COUNTIF($B$2:$B$1000,B2)=1</formula1>
     </dataValidation>
   </dataValidations>
-  <conditionalFormatting sqref="B2:B1000">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>COUNTIF($B$2:$B$1000,B2)&gt;1</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: output unik across sheets - kode hanya boleh keluar sekali (Agus XOR Rexa) dan tidak duplikat per sheet
</commit_message>
<xml_diff>
--- a/Sistem_Keluar_Masuk_Barang.xlsx
+++ b/Sistem_Keluar_Masuk_Barang.xlsx
@@ -18207,9 +18207,14 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B1000">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND(B2&lt;&gt;"",NOT(AND(COUNTIF('Input Barang'!$B$2:$B$1000,B2)&gt;=1,COUNTIF($B$2:$B$1000,B2)&lt;=1,COUNTIF('Output Rexa'!$B$2:$B$1000,B2)=0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="0" showErrorMessage="1" errorStyle="stop" errorTitle="Kode Tidak Terdaftar" error="Kode barang ini TIDAK ADA di sheet Input Barang. Input dulu di sheet Input Barang." sqref="B2:B1000">
-      <formula1>COUNTIF('Input Barang'!$B$2:$B$1000,B2)&gt;=1</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="0" showErrorMessage="1" errorStyle="stop" errorTitle="Kode Tidak Valid" error="Kode ditolak. Kemungkinan: (1) kode tidak ada di sheet Input Barang, (2) kode sudah discan di sheet ini, atau (3) kode sudah discan di sheet Output Rexa." sqref="B2:B1000">
+      <formula1>AND(COUNTIF('Input Barang'!$B$2:$B$1000,B2)&gt;=1,COUNTIF($B$2:$B$1000,B2)&lt;=1,COUNTIF('Output Rexa'!$B$2:$B$1000,B2)=0)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -27229,9 +27234,14 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B1000">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND(B2&lt;&gt;"",NOT(AND(COUNTIF('Input Barang'!$B$2:$B$1000,B2)&gt;=1,COUNTIF($B$2:$B$1000,B2)&lt;=1,COUNTIF('Output Agus'!$B$2:$B$1000,B2)=0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="0" showErrorMessage="1" errorStyle="stop" errorTitle="Kode Tidak Terdaftar" error="Kode barang ini TIDAK ADA di sheet Input Barang. Input dulu di sheet Input Barang." sqref="B2:B1000">
-      <formula1>COUNTIF('Input Barang'!$B$2:$B$1000,B2)&gt;=1</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="0" showErrorMessage="1" errorStyle="stop" errorTitle="Kode Tidak Valid" error="Kode ditolak. Kemungkinan: (1) kode tidak ada di sheet Input Barang, (2) kode sudah discan di sheet ini, atau (3) kode sudah discan di sheet Output Agus." sqref="B2:B1000">
+      <formula1>AND(COUNTIF('Input Barang'!$B$2:$B$1000,B2)&gt;=1,COUNTIF($B$2:$B$1000,B2)&lt;=1,COUNTIF('Output Agus'!$B$2:$B$1000,B2)=0)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>